<commit_message>
Updated the buildSchedule to initiate correct processes in startYear
</commit_message>
<xml_diff>
--- a/documentation/SimPathsUK_Schedule.xlsx
+++ b/documentation/SimPathsUK_Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsUK_refactored/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D93502D-C4B6-AF47-8595-00D326E99338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C065F163-668D-F045-9F05-83D3C93947A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-29920" yWindow="3940" windowWidth="29180" windowHeight="18880" xr2:uid="{D5C64B29-9946-AF44-8A1E-67952110700F}"/>
   </bookViews>
@@ -477,6 +477,15 @@
     <t>reg_eq5d.xlsx</t>
   </si>
   <si>
+    <t>S2a, S2b, S2c, S2d, S2e</t>
+  </si>
+  <si>
+    <t>S3a, S3b, S3c, S3d</t>
+  </si>
+  <si>
+    <t>//currently does not impact the model but is kept for future development</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">demLifeSatEQ5D </t>
     </r>
@@ -487,17 +496,8 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t>is NOT present in InitPop,so I would keep this process called in the startYear</t>
+      <t>is NOT present in InitPop,so the process is kept in the startYear</t>
     </r>
-  </si>
-  <si>
-    <t>S2a, S2b, S2c, S2d, S2e</t>
-  </si>
-  <si>
-    <t>S3a, S3b, S3c, S3d</t>
-  </si>
-  <si>
-    <t>//not much used but is kep for future development</t>
   </si>
 </sst>
 </file>
@@ -540,7 +540,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -555,18 +555,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
+        <fgColor theme="3" tint="0.749992370372631"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -891,11 +885,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -935,17 +938,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -969,15 +964,61 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -987,72 +1028,26 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1394,7 +1389,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EB35C93-5050-2740-9B24-47F315D2BE07}">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.83203125" style="11" customWidth="1"/>
@@ -1423,152 +1418,152 @@
       <c r="E1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="28" t="s">
+      <c r="F1" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="G1" s="37" t="s">
+      <c r="G1" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="H1" s="30" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A2" s="63">
+      <c r="A2" s="46">
         <v>1</v>
       </c>
-      <c r="B2" s="64" t="s">
+      <c r="B2" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="65" t="s">
+      <c r="D2" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="39" t="s">
+      <c r="E2" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="66"/>
-      <c r="G2" s="39"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="34"/>
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="63">
+      <c r="A3" s="46">
         <v>2</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="39" t="s">
+      <c r="D3" s="47"/>
+      <c r="E3" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="66"/>
-      <c r="G3" s="39"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="34"/>
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="63">
+      <c r="A4" s="46">
         <v>3</v>
       </c>
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="64"/>
-      <c r="E4" s="39" t="s">
+      <c r="D4" s="47"/>
+      <c r="E4" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="66"/>
-      <c r="G4" s="39"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="34"/>
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="77">
+      <c r="A5" s="58">
         <v>4</v>
       </c>
-      <c r="B5" s="78" t="s">
+      <c r="B5" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="79" t="s">
-        <v>105</v>
-      </c>
-      <c r="D5" s="78"/>
-      <c r="E5" s="79" t="s">
+      <c r="C5" s="60" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="59"/>
+      <c r="E5" s="60" t="s">
         <v>109</v>
       </c>
-      <c r="F5" s="80"/>
-      <c r="G5" s="79"/>
+      <c r="F5" s="61"/>
+      <c r="G5" s="60"/>
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="77">
+      <c r="A6" s="58">
         <v>5</v>
       </c>
-      <c r="B6" s="78" t="s">
+      <c r="B6" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="79" t="s">
-        <v>105</v>
-      </c>
-      <c r="D6" s="78"/>
-      <c r="E6" s="79" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="80"/>
-      <c r="G6" s="79"/>
+      <c r="C6" s="60" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="59"/>
+      <c r="E6" s="60" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="61"/>
+      <c r="G6" s="60"/>
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A7" s="25">
+      <c r="A7" s="21">
         <v>6</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="D7" s="27" t="s">
+      <c r="C7" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="E7" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" s="29" t="s">
+      <c r="E7" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="22" t="s">
         <v>108</v>
       </c>
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="45">
+      <c r="A8" s="16">
         <v>7</v>
       </c>
-      <c r="B8" s="46" t="s">
+      <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="D8" s="46" t="s">
+      <c r="C8" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="46" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" s="47" t="s">
+      <c r="E8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="G8" s="46" t="s">
+      <c r="G8" s="2" t="s">
         <v>75</v>
       </c>
       <c r="H8" s="4"/>
@@ -1589,7 +1584,7 @@
       <c r="E9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="21" t="s">
+      <c r="F9" s="18" t="s">
         <v>119</v>
       </c>
       <c r="G9" s="2" t="s">
@@ -1611,32 +1606,32 @@
       <c r="E10" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="30" t="s">
+      <c r="F10" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="G10" s="39"/>
+      <c r="G10" s="34"/>
       <c r="H10" s="4"/>
     </row>
     <row r="11" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A11" s="45">
+      <c r="A11" s="16">
         <v>10</v>
       </c>
-      <c r="B11" s="46" t="s">
+      <c r="B11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="D11" s="48" t="s">
+      <c r="C11" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="E11" s="46" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="47" t="s">
+      <c r="E11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="G11" s="46" t="s">
+      <c r="G11" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H11" s="4"/>
@@ -1655,10 +1650,10 @@
       <c r="E12" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="30" t="s">
+      <c r="F12" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="G12" s="39"/>
+      <c r="G12" s="34"/>
       <c r="H12" s="4"/>
     </row>
     <row r="13" spans="1:8" ht="17" x14ac:dyDescent="0.2">
@@ -1677,7 +1672,7 @@
       <c r="E13" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F13" s="21" t="s">
+      <c r="F13" s="18" t="s">
         <v>120</v>
       </c>
       <c r="G13" s="2" t="s">
@@ -1698,10 +1693,10 @@
       <c r="D14" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F14" s="22" t="s">
+      <c r="E14" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="19" t="s">
         <v>122</v>
       </c>
       <c r="G14" s="2" t="s">
@@ -1725,7 +1720,7 @@
       <c r="E15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F15" s="31" t="s">
+      <c r="F15" s="27" t="s">
         <v>123</v>
       </c>
       <c r="G15" s="3" t="s">
@@ -1734,23 +1729,23 @@
       <c r="H15" s="4"/>
     </row>
     <row r="16" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="40">
+      <c r="A16" s="62">
         <v>15</v>
       </c>
-      <c r="B16" s="41" t="s">
+      <c r="B16" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="41" t="s">
-        <v>105</v>
-      </c>
-      <c r="D16" s="41"/>
-      <c r="E16" s="42" t="s">
+      <c r="C16" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="D16" s="63"/>
+      <c r="E16" s="64" t="s">
         <v>20</v>
       </c>
-      <c r="F16" s="43" t="s">
+      <c r="F16" s="65" t="s">
         <v>115</v>
       </c>
-      <c r="G16" s="44" t="s">
+      <c r="G16" s="66" t="s">
         <v>129</v>
       </c>
       <c r="H16" s="4"/>
@@ -1768,10 +1763,10 @@
       <c r="D17" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E17" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F17" s="22" t="s">
+      <c r="E17" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="19" t="s">
         <v>124</v>
       </c>
       <c r="G17" s="2" t="s">
@@ -1792,10 +1787,10 @@
       <c r="D18" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E18" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F18" s="22"/>
+      <c r="E18" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="19"/>
       <c r="G18" s="2"/>
       <c r="H18" s="4"/>
     </row>
@@ -1815,26 +1810,26 @@
       <c r="E19" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F19" s="21"/>
+      <c r="F19" s="18"/>
       <c r="G19" s="2"/>
       <c r="H19" s="4"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="16">
+      <c r="A20" s="62">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2" t="s">
+      <c r="C20" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="D20" s="63"/>
+      <c r="E20" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="F20" s="21"/>
-      <c r="G20" s="2"/>
+      <c r="F20" s="70"/>
+      <c r="G20" s="63"/>
       <c r="H20" s="4"/>
     </row>
     <row r="21" spans="1:8" ht="17" x14ac:dyDescent="0.2">
@@ -1850,10 +1845,10 @@
       <c r="D21" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E21" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F21" s="22" t="s">
+      <c r="E21" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F21" s="19" t="s">
         <v>125</v>
       </c>
       <c r="G21" s="2" t="s">
@@ -1874,168 +1869,168 @@
       <c r="D22" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="E22" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F22" s="22"/>
+      <c r="E22" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" s="19"/>
       <c r="G22" s="7"/>
-      <c r="H22" s="24" t="s">
+      <c r="H22" s="20" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A23" s="45">
+      <c r="A23" s="16">
         <v>22</v>
       </c>
-      <c r="B23" s="46" t="s">
+      <c r="B23" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="D23" s="48" t="s">
+      <c r="C23" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E23" s="46" t="s">
-        <v>21</v>
-      </c>
-      <c r="F23" s="47" t="s">
+      <c r="E23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="G23" s="48" t="s">
+      <c r="G23" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="H23" s="4"/>
+    </row>
+    <row r="24" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A24" s="16">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="H23" s="4"/>
-    </row>
-    <row r="24" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="45">
-        <v>23</v>
-      </c>
-      <c r="B24" s="46" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="D24" s="48" t="s">
-        <v>71</v>
-      </c>
-      <c r="E24" s="46" t="s">
-        <v>21</v>
-      </c>
-      <c r="F24" s="47" t="s">
-        <v>126</v>
-      </c>
-      <c r="G24" s="46" t="s">
+      <c r="H24" s="4"/>
+    </row>
+    <row r="25" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A25" s="37">
+        <v>24</v>
+      </c>
+      <c r="B25" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="35" t="s">
+        <v>105</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="E25" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="F25" s="36"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="40" t="s">
         <v>138</v>
       </c>
-      <c r="H24" s="4"/>
-    </row>
-    <row r="25" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A25" s="51">
-        <v>24</v>
-      </c>
-      <c r="B25" s="49" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" s="49" t="s">
-        <v>105</v>
-      </c>
-      <c r="D25" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="E25" s="49" t="s">
-        <v>21</v>
-      </c>
-      <c r="F25" s="50"/>
-      <c r="G25" s="53"/>
-      <c r="H25" s="54" t="s">
-        <v>139</v>
-      </c>
     </row>
     <row r="26" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="45">
+      <c r="A26" s="16">
         <v>25</v>
       </c>
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="48" t="s">
-        <v>105</v>
-      </c>
-      <c r="D26" s="48" t="s">
+      <c r="C26" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E26" s="46" t="s">
+      <c r="E26" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F26" s="55" t="s">
+      <c r="F26" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="G26" s="48" t="s">
+      <c r="G26" s="3" t="s">
         <v>86</v>
       </c>
       <c r="H26" s="4"/>
     </row>
     <row r="27" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A27" s="45">
+      <c r="A27" s="16">
         <v>26</v>
       </c>
-      <c r="B27" s="46" t="s">
+      <c r="B27" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="D27" s="48" t="s">
+      <c r="C27" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E27" s="46" t="s">
+      <c r="E27" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F27" s="47"/>
-      <c r="G27" s="46"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="2"/>
       <c r="H27" s="4"/>
     </row>
     <row r="28" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A28" s="45">
+      <c r="A28" s="16">
         <v>27</v>
       </c>
-      <c r="B28" s="46" t="s">
+      <c r="B28" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="D28" s="48" t="s">
+      <c r="C28" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="E28" s="46" t="s">
-        <v>21</v>
-      </c>
-      <c r="F28" s="47"/>
-      <c r="G28" s="46"/>
-      <c r="H28" s="56"/>
+      <c r="E28" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" s="18"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="41"/>
     </row>
     <row r="29" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A29" s="45">
+      <c r="A29" s="16">
         <v>28</v>
       </c>
-      <c r="B29" s="46" t="s">
+      <c r="B29" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C29" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="D29" s="48" t="s">
+      <c r="C29" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E29" s="46" t="s">
+      <c r="E29" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F29" s="47"/>
-      <c r="G29" s="46"/>
-      <c r="H29" s="56"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="41"/>
     </row>
     <row r="30" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="16">
@@ -2050,13 +2045,13 @@
       <c r="D30" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="E30" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F30" s="32" t="s">
+      <c r="E30" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="G30" s="38" t="s">
+      <c r="G30" s="33" t="s">
         <v>128</v>
       </c>
       <c r="H30" s="4"/>
@@ -2074,10 +2069,10 @@
       <c r="D31" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E31" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F31" s="33" t="s">
+      <c r="E31" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F31" s="29" t="s">
         <v>133</v>
       </c>
       <c r="G31" s="3" t="s">
@@ -2098,10 +2093,10 @@
       <c r="D32" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E32" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F32" s="22" t="s">
+      <c r="E32" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F32" s="19" t="s">
         <v>131</v>
       </c>
       <c r="G32" s="2" t="s">
@@ -2109,7 +2104,7 @@
       </c>
       <c r="H32" s="4"/>
     </row>
-    <row r="33" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="16">
         <v>32</v>
       </c>
@@ -2122,10 +2117,10 @@
       <c r="D33" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="E33" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F33" s="22" t="s">
+      <c r="E33" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F33" s="19" t="s">
         <v>131</v>
       </c>
       <c r="G33" s="2" t="s">
@@ -2133,7 +2128,7 @@
       </c>
       <c r="H33" s="4"/>
     </row>
-    <row r="34" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="16">
         <v>33</v>
       </c>
@@ -2146,10 +2141,10 @@
       <c r="D34" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="E34" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F34" s="22" t="s">
+      <c r="E34" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F34" s="19" t="s">
         <v>131</v>
       </c>
       <c r="G34" s="2" t="s">
@@ -2157,7 +2152,7 @@
       </c>
       <c r="H34" s="4"/>
     </row>
-    <row r="35" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A35" s="16">
         <v>34</v>
       </c>
@@ -2170,10 +2165,10 @@
       <c r="D35" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E35" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F35" s="33" t="s">
+      <c r="E35" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" s="29" t="s">
         <v>134</v>
       </c>
       <c r="G35" s="3" t="s">
@@ -2181,7 +2176,7 @@
       </c>
       <c r="H35" s="4"/>
     </row>
-    <row r="36" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A36" s="16">
         <v>35</v>
       </c>
@@ -2194,10 +2189,10 @@
       <c r="D36" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E36" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F36" s="33" t="s">
+      <c r="E36" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F36" s="29" t="s">
         <v>134</v>
       </c>
       <c r="G36" s="3" t="s">
@@ -2205,7 +2200,7 @@
       </c>
       <c r="H36" s="4"/>
     </row>
-    <row r="37" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A37" s="16">
         <v>36</v>
       </c>
@@ -2218,10 +2213,10 @@
       <c r="D37" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E37" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F37" s="33" t="s">
+      <c r="E37" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F37" s="29" t="s">
         <v>134</v>
       </c>
       <c r="G37" s="3" t="s">
@@ -2229,7 +2224,7 @@
       </c>
       <c r="H37" s="4"/>
     </row>
-    <row r="38" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="16">
         <v>37</v>
       </c>
@@ -2242,10 +2237,10 @@
       <c r="D38" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E38" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F38" s="22" t="s">
+      <c r="E38" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F38" s="19" t="s">
         <v>132</v>
       </c>
       <c r="G38" s="2" t="s">
@@ -2253,7 +2248,7 @@
       </c>
       <c r="H38" s="4"/>
     </row>
-    <row r="39" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="16">
         <v>38</v>
       </c>
@@ -2266,10 +2261,10 @@
       <c r="D39" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E39" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F39" s="22" t="s">
+      <c r="E39" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F39" s="19" t="s">
         <v>132</v>
       </c>
       <c r="G39" s="2" t="s">
@@ -2277,7 +2272,7 @@
       </c>
       <c r="H39" s="4"/>
     </row>
-    <row r="40" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="16">
         <v>39</v>
       </c>
@@ -2290,10 +2285,10 @@
       <c r="D40" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E40" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F40" s="22" t="s">
+      <c r="E40" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F40" s="19" t="s">
         <v>132</v>
       </c>
       <c r="G40" s="3" t="s">
@@ -2301,165 +2296,170 @@
       </c>
       <c r="H40" s="4"/>
     </row>
-    <row r="41" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A41" s="40">
+    <row r="41" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A41" s="15">
         <v>40</v>
       </c>
-      <c r="B41" s="41" t="s">
+      <c r="B41" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C41" s="41" t="s">
-        <v>105</v>
-      </c>
-      <c r="D41" s="44" t="s">
+      <c r="C41" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D41" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="E41" s="41" t="s">
-        <v>21</v>
-      </c>
-      <c r="F41" s="75" t="s">
+      <c r="E41" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F41" s="67" t="s">
         <v>101</v>
       </c>
-      <c r="G41" s="76"/>
+      <c r="G41" s="34"/>
       <c r="H41" s="4"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="40">
+      <c r="I41" s="78"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A42" s="62">
         <v>41</v>
       </c>
-      <c r="B42" s="41" t="s">
+      <c r="B42" s="63" t="s">
         <v>51</v>
       </c>
-      <c r="C42" s="41" t="s">
-        <v>105</v>
-      </c>
-      <c r="D42" s="41"/>
-      <c r="E42" s="41" t="s">
+      <c r="C42" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="D42" s="63"/>
+      <c r="E42" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="F42" s="57" t="s">
+      <c r="F42" s="68" t="s">
         <v>102</v>
       </c>
-      <c r="G42" s="58"/>
-      <c r="H42" s="4"/>
-    </row>
-    <row r="43" spans="1:8" ht="52" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="17">
+      <c r="G42" s="69"/>
+      <c r="H42" s="75"/>
+      <c r="I42" s="78"/>
+      <c r="J42" s="77"/>
+    </row>
+    <row r="43" spans="1:10" ht="52" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="71">
         <v>42</v>
       </c>
-      <c r="B43" s="18" t="s">
+      <c r="B43" s="72" t="s">
         <v>52</v>
       </c>
-      <c r="C43" s="18" t="s">
+      <c r="C43" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="D43" s="19" t="s">
+      <c r="D43" s="73" t="s">
         <v>98</v>
       </c>
-      <c r="E43" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="F43" s="23" t="s">
+      <c r="E43" s="72" t="s">
+        <v>21</v>
+      </c>
+      <c r="F43" s="74" t="s">
         <v>135</v>
       </c>
-      <c r="G43" s="18" t="s">
+      <c r="G43" s="72" t="s">
         <v>99</v>
       </c>
-      <c r="H43" s="35" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A44" s="59">
+      <c r="H43" s="76" t="s">
+        <v>139</v>
+      </c>
+      <c r="I43" s="78"/>
+      <c r="J43" s="77"/>
+    </row>
+    <row r="44" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+      <c r="A44" s="42">
         <v>43</v>
       </c>
-      <c r="B44" s="60" t="s">
+      <c r="B44" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="C44" s="38" t="s">
-        <v>105</v>
-      </c>
-      <c r="D44" s="61" t="s">
+      <c r="C44" s="33" t="s">
+        <v>105</v>
+      </c>
+      <c r="D44" s="44" t="s">
         <v>100</v>
       </c>
-      <c r="E44" s="38" t="s">
+      <c r="E44" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="F44" s="62"/>
-      <c r="G44" s="38"/>
+      <c r="F44" s="45"/>
+      <c r="G44" s="33"/>
       <c r="H44" s="4"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A45" s="67">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A45" s="50">
         <v>44</v>
       </c>
-      <c r="B45" s="68" t="s">
+      <c r="B45" s="51" t="s">
         <v>54</v>
       </c>
-      <c r="C45" s="69" t="s">
+      <c r="C45" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="D45" s="68"/>
-      <c r="E45" s="69" t="s">
+      <c r="D45" s="51"/>
+      <c r="E45" s="52" t="s">
         <v>110</v>
       </c>
-      <c r="F45" s="70"/>
-      <c r="G45" s="69"/>
+      <c r="F45" s="53"/>
+      <c r="G45" s="52"/>
       <c r="H45" s="4"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A46" s="67">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A46" s="50">
         <v>45</v>
       </c>
-      <c r="B46" s="68" t="s">
+      <c r="B46" s="51" t="s">
         <v>55</v>
       </c>
-      <c r="C46" s="69" t="s">
+      <c r="C46" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="D46" s="68"/>
-      <c r="E46" s="69" t="s">
-        <v>21</v>
-      </c>
-      <c r="F46" s="70"/>
-      <c r="G46" s="69"/>
+      <c r="D46" s="51"/>
+      <c r="E46" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="F46" s="53"/>
+      <c r="G46" s="52"/>
       <c r="H46" s="4"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A47" s="67">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A47" s="50">
         <v>46</v>
       </c>
-      <c r="B47" s="68" t="s">
+      <c r="B47" s="51" t="s">
         <v>56</v>
       </c>
-      <c r="C47" s="69" t="s">
+      <c r="C47" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="D47" s="68"/>
-      <c r="E47" s="69" t="s">
+      <c r="D47" s="51"/>
+      <c r="E47" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="F47" s="70"/>
-      <c r="G47" s="69"/>
+      <c r="F47" s="53"/>
+      <c r="G47" s="52"/>
       <c r="H47" s="4"/>
     </row>
-    <row r="48" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="71">
+    <row r="48" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="54">
         <v>47</v>
       </c>
-      <c r="B48" s="72" t="s">
+      <c r="B48" s="55" t="s">
         <v>57</v>
       </c>
-      <c r="C48" s="73" t="s">
+      <c r="C48" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="D48" s="72"/>
-      <c r="E48" s="73" t="s">
+      <c r="D48" s="55"/>
+      <c r="E48" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="F48" s="74"/>
-      <c r="G48" s="73"/>
-      <c r="H48" s="36"/>
+      <c r="F48" s="57"/>
+      <c r="G48" s="56"/>
+      <c r="H48" s="31"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>